<commit_message>
updation in server code and in CSV file too
</commit_message>
<xml_diff>
--- a/data/submissions.xlsx
+++ b/data/submissions.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -467,9 +467,26 @@
         <v>DEEPA</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>2026-08-27T05:53:18.588Z</v>
+      </c>
+      <c r="B5" t="str">
+        <v>sbbfuels-attendance</v>
+      </c>
+      <c r="C5" t="str">
+        <v>rishiraj@sbbfuels.com</v>
+      </c>
+      <c r="D5" t="str">
+        <v>vasA</v>
+      </c>
+      <c r="E5" t="str">
+        <v>werd</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Updated the server file include delected function
</commit_message>
<xml_diff>
--- a/data/submissions.xlsx
+++ b/data/submissions.xlsx
@@ -31,28 +31,43 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
+  <numFmts count="0"/>
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
+      <sz val="11"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <color rgb="FF0000"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill patternType="none">
+        <bgColor/>
+      </patternFill>
     </fill>
     <fill>
-      <patternFill patternType="gray125"/>
+      <patternFill patternType="gray125">
+        <bgColor/>
+      </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
     <border>
       <left/>
       <right/>
@@ -61,13 +76,16 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="4">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -397,96 +415,167 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:H6"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="str">
+      <c r="A1" s="2" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" s="2" t="str">
         <v>timestamp</v>
       </c>
-      <c r="B1" t="str">
+      <c r="C1" s="2" t="str">
         <v>name</v>
       </c>
-      <c r="C1" t="str">
+      <c r="D1" s="2" t="str">
         <v>email</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" s="2" t="str">
         <v>subject</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" s="2" t="str">
         <v>message</v>
+      </c>
+      <c r="G1" s="2" t="str">
+        <v>status</v>
+      </c>
+      <c r="H1" s="2" t="str">
+        <v>deletedAt</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="str">
+      <c r="A2" s="3" t="str">
+        <v>legacy-0-2026-08-25T11:58:50.900Z</v>
+      </c>
+      <c r="B2" s="3" t="str">
         <v>2026-08-25T11:58:50.900Z</v>
       </c>
-      <c r="B2" t="str">
+      <c r="C2" s="3" t="str">
         <v>rishir</v>
       </c>
-      <c r="C2" t="str">
+      <c r="D2" s="3" t="str">
         <v>FBuoiare@gmail.com</v>
       </c>
-      <c r="D2" t="str">
+      <c r="E2" s="3" t="str">
         <v>fuwbacd</v>
       </c>
-      <c r="E2" t="str">
+      <c r="F2" s="3" t="str">
         <v>scdhbvkcuya</v>
+      </c>
+      <c r="G2" s="3" t="str">
+        <v>Deleted</v>
+      </c>
+      <c r="H2" s="3" t="str">
+        <v>2026-09-03T07:18:01.162Z</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="str">
+      <c r="A3" s="3" t="str">
+        <v>legacy-1-2026-08-25T12:06:34.426Z</v>
+      </c>
+      <c r="B3" s="3" t="str">
         <v>2026-08-25T12:06:34.426Z</v>
       </c>
-      <c r="B3" t="str">
+      <c r="C3" s="3" t="str">
         <v>Rishi Raj Sharma</v>
       </c>
-      <c r="C3" t="str">
+      <c r="D3" s="3" t="str">
         <v>rishiraj@sbbfuels.com</v>
       </c>
-      <c r="D3" t="str">
+      <c r="E3" s="3" t="str">
         <v>fwew</v>
       </c>
-      <c r="E3" t="str">
+      <c r="F3" s="3" t="str">
         <v>WFE</v>
+      </c>
+      <c r="G3" s="3" t="str">
+        <v>Deleted</v>
+      </c>
+      <c r="H3" s="3" t="str">
+        <v>2026-09-03T07:18:08.054Z</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="str">
+      <c r="A4" s="3" t="str">
+        <v>legacy-2-2026-08-25T12:06:56.365Z</v>
+      </c>
+      <c r="B4" s="3" t="str">
         <v>2026-08-25T12:06:56.365Z</v>
       </c>
-      <c r="B4" t="str">
+      <c r="C4" s="3" t="str">
         <v>Rishi Raj Sharma</v>
       </c>
-      <c r="C4" t="str">
+      <c r="D4" s="3" t="str">
         <v>rishiraj@sbbfuels.com</v>
       </c>
-      <c r="D4" t="str">
+      <c r="E4" s="3" t="str">
         <v>VDA</v>
       </c>
-      <c r="E4" t="str">
+      <c r="F4" s="3" t="str">
         <v>DEEPA</v>
+      </c>
+      <c r="G4" s="3" t="str">
+        <v>Deleted</v>
+      </c>
+      <c r="H4" s="3" t="str">
+        <v>2026-09-03T07:18:11.041Z</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="str">
+      <c r="A5" s="2" t="str">
+        <v>legacy-3-2026-08-27T05:53:18.588Z</v>
+      </c>
+      <c r="B5" s="2" t="str">
         <v>2026-08-27T05:53:18.588Z</v>
       </c>
-      <c r="B5" t="str">
+      <c r="C5" s="2" t="str">
         <v>sbbfuels-attendance</v>
       </c>
-      <c r="C5" t="str">
+      <c r="D5" s="2" t="str">
         <v>rishiraj@sbbfuels.com</v>
       </c>
-      <c r="D5" t="str">
+      <c r="E5" s="2" t="str">
         <v>vasA</v>
       </c>
-      <c r="E5" t="str">
+      <c r="F5" s="2" t="str">
         <v>werd</v>
+      </c>
+      <c r="G5" s="2" t="str">
+        <v>Active</v>
+      </c>
+      <c r="H5" s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="str">
+        <v>75b64355-a282-42b1-b36e-6b9282523af6</v>
+      </c>
+      <c r="B6" s="2" t="str">
+        <v>2026-09-03T07:17:45.767Z</v>
+      </c>
+      <c r="C6" s="2" t="str">
+        <v>Rishiraj</v>
+      </c>
+      <c r="D6" s="2" t="str">
+        <v>rishi@gmail.com</v>
+      </c>
+      <c r="E6" s="2" t="str">
+        <v>DDGS</v>
+      </c>
+      <c r="F6" s="2" t="str">
+        <v>I want that for my poultry farm</v>
+      </c>
+      <c r="G6" s="2" t="str">
+        <v>Active</v>
+      </c>
+      <c r="H6" s="2" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>